<commit_message>
v2: rebuild task after Gemini solved v1 at ~100%
Trajectory 6 (gemini-3.5-flash) scored ~100% on v1: it wrote Python and computed
every value, including the drop-side fault meant to defeat it. Arithmetic volume
is not difficulty for a model with a code interpreter.

v2 moves the difficulty into deciding what to compute:

- FCN-2291 reroutes Leg C after the as-built survey closed. Ignoring it
  understates Leg C design loss by 1.53 dB and falsely flags three healthy
  subscribers as faults.
- The 1:8 splitter is certified per port, not nominal. Each leg draws from a
  different port; a nominal 10.50 dB makes all 16 rows wrong.
- Remediation ranks on SLA credit exposure, not headcount, so a single
  Business 10G subscriber outranks a leg of three.

Fifth input file (the change notice, .docx). Standard bumped to Rev E.
</commit_message>
<xml_diff>
--- a/task36/attachments/ONT_Power_Survey_FDH14.xlsx
+++ b/task36/attachments/ONT_Power_Survey_FDH14.xlsx
@@ -466,7 +466,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,7 +542,7 @@
         <v>120</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-22.65</v>
+        <v>-22.5</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
         <v>185</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>-22.86</v>
+        <v>-22.71</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
         <v>240</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>-22.72</v>
+        <v>-22.57</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
@@ -626,7 +626,7 @@
         <v>95</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>-25.66</v>
+        <v>-25.78</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
@@ -654,11 +654,11 @@
         <v>160</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>-25.79</v>
+        <v>-25.91</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Business 2G</t>
+          <t>Residential 1G</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
         <v>225</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>-25.67</v>
+        <v>-25.79</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
         <v>310</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>-25.8</v>
+        <v>-25.92</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
         <v>140</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>-23</v>
+        <v>-24.47</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
@@ -766,7 +766,7 @@
         <v>205</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>-23.15</v>
+        <v>-24.61</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
@@ -794,11 +794,11 @@
         <v>95</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>-26.28</v>
+        <v>-27.74</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Business 2G</t>
+          <t>Business 10G Priority</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
         <v>270</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>-23.04</v>
+        <v>-24.51</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>110</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>-27.08</v>
+        <v>-27.39</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
@@ -878,11 +878,11 @@
         <v>175</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>-27.21</v>
+        <v>-27.52</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Business 2G</t>
+          <t>Residential 1G</t>
         </is>
       </c>
     </row>
@@ -906,11 +906,11 @@
         <v>250</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>-27.17</v>
+        <v>-27.48</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Business 2G</t>
+          <t>Residential 1G</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
         <v>130</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>-22.85</v>
+        <v>-22.63</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         <v>195</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>-23</v>
+        <v>-22.78</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>

</xml_diff>